<commit_message>
added stock summary report
</commit_message>
<xml_diff>
--- a/User files/Sales/GLAMORISE_Update Greige_13.8.2026.xlsx
+++ b/User files/Sales/GLAMORISE_Update Greige_13.8.2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Claude\Eschler\User files\Sales\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\it\Desktop\workspace\Eschler\User files\Sales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EE191E30-09ED-4938-BF4D-40267846B8B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD78CEC9-191F-4F9B-B31E-F5CCACA28E47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="811" xr2:uid="{9F1F87CC-15C7-4136-B520-189C0441DDFC}"/>
   </bookViews>
@@ -36,19 +36,10 @@
     <definedName name="_xlnm.Print_Area" localSheetId="1">'2943_IAY-076AA.11'!$A$1:$Q$85</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'2975_IAY-077AA.11'!$A$1:$Q$20</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>

</xml_diff>